<commit_message>
Netforvaltning Sundhed har fået status Godkendt for afsendelse af BIN01
</commit_message>
<xml_diff>
--- a/html/Specialsystemer_excel.XLSX
+++ b/html/Specialsystemer_excel.XLSX
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0011DAB5-DCF0-44A8-8329-7AEB1004490E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4B5F295-6238-46A5-AF8A-F60EEA94375D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1101" uniqueCount="234">
   <si>
     <t>Standard</t>
   </si>
@@ -1309,6 +1309,9 @@
       <c r="AH4" t="s">
         <v>62</v>
       </c>
+      <c r="AN4" t="s">
+        <v>62</v>
+      </c>
       <c r="AO4" t="s">
         <v>62</v>
       </c>

</xml_diff>